<commit_message>
TODOS ARQUIVOS - DIARIO_CLASSE
PRECISA SER ANALISADOS PARA VER SE AS INFORMAÇÕES ESTÃO BATENDO COM OS DADOS QUE ESTÃO NO SISTEMA
</commit_message>
<xml_diff>
--- a/AEE.xlsx
+++ b/AEE.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Planilha1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="HTML_1" vbProcedure="false">Planilha1!$A$1:$T$71</definedName>
-    <definedName function="false" hidden="false" name="HTML_all" vbProcedure="false">Planilha1!$A$1:$T$71</definedName>
+    <definedName function="false" hidden="false" name="HTML_1" vbProcedure="false">Planilha1!$A$1:$T$72</definedName>
+    <definedName function="false" hidden="false" name="HTML_all" vbProcedure="false">Planilha1!$A$1:$T$72</definedName>
     <definedName function="false" hidden="false" name="HTML_tables" vbProcedure="false">#REF!</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="241">
   <si>
     <t xml:space="preserve">Nº classe</t>
   </si>
@@ -183,6 +183,21 @@
     <t xml:space="preserve">TRAVESSA SÃO TIAGO - 80, PARQUE CAPUAVA - SANTO ANDRE - SP</t>
   </si>
   <si>
+    <t xml:space="preserve">ANTHONY VIANA SILVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/03/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28/05/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINDROME DE DOWN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUA CORINA MAGGINI - 595, TAMANDUATEÍ 8 - SANTO ANDRE - SP</t>
+  </si>
+  <si>
     <t xml:space="preserve">ALICIA RODRIGUES DOS SANTOS SILVA</t>
   </si>
   <si>
@@ -391,9 +406,6 @@
   </si>
   <si>
     <t xml:space="preserve">03/09/2018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SINDROME DE DOWN</t>
   </si>
   <si>
     <t xml:space="preserve">RUA ARMANDO SETTI - 41, PARQUE CAPUAVA - SANTO ANDRE - SP</t>
@@ -951,7 +963,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T71"/>
+  <dimension ref="A1:T72"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1396,7 +1408,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
-        <v>300747282</v>
+        <v>300747281</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>20</v>
@@ -1405,16 +1417,16 @@
         <v>0</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>52</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>124188843</v>
+        <v>125754632</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>22</v>
@@ -1423,7 +1435,7 @@
         <v>53</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>25</v>
@@ -1435,14 +1447,14 @@
         <v>27</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="T9" s="1" t="s">
         <v>30</v>
@@ -1459,22 +1471,22 @@
         <v>0</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>123050338</v>
+        <v>124188843</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>24</v>
@@ -1489,14 +1501,14 @@
         <v>27</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>30</v>
@@ -1513,25 +1525,25 @@
         <v>0</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>123898781</v>
+        <v>123050338</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>25</v>
@@ -1543,7 +1555,7 @@
         <v>27</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
@@ -1558,7 +1570,7 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
-        <v>300747283</v>
+        <v>300747282</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>20</v>
@@ -1567,16 +1579,16 @@
         <v>0</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>64</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>126207007</v>
+        <v>123898781</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>22</v>
@@ -1585,7 +1597,7 @@
         <v>65</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>25</v>
@@ -1597,14 +1609,14 @@
         <v>27</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>41</v>
+        <v>67</v>
       </c>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="T12" s="1" t="s">
         <v>30</v>
@@ -1621,22 +1633,22 @@
         <v>0</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>122323450</v>
+        <v>126207007</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>24</v>
@@ -1651,14 +1663,14 @@
         <v>27</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="T13" s="1" t="s">
         <v>30</v>
@@ -1675,22 +1687,22 @@
         <v>0</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>124386580</v>
+        <v>122323450</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>24</v>
@@ -1712,7 +1724,7 @@
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
       <c r="S14" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>30</v>
@@ -1729,22 +1741,22 @@
         <v>0</v>
       </c>
       <c r="D15" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>124386580</v>
+      </c>
+      <c r="G15" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F15" s="1" t="n">
-        <v>122428809</v>
-      </c>
-      <c r="G15" s="1" t="n">
-        <v>9</v>
-      </c>
       <c r="H15" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>24</v>
@@ -1759,14 +1771,14 @@
         <v>27</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="T15" s="1" t="s">
         <v>30</v>
@@ -1783,34 +1795,34 @@
         <v>0</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>124197224</v>
+        <v>122428809</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>79</v>
+        <v>26</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="N16" s="1" t="s">
         <v>28</v>
@@ -1820,7 +1832,7 @@
       <c r="Q16" s="1"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="T16" s="1" t="s">
         <v>30</v>
@@ -1837,44 +1849,44 @@
         <v>0</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" s="1" t="n">
+        <v>124197224</v>
+      </c>
+      <c r="G17" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="F17" s="1" t="n">
-        <v>125011562</v>
-      </c>
-      <c r="G17" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I17" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="J17" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="K17" s="2" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>27</v>
+        <v>85</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="T17" s="1" t="s">
         <v>30</v>
@@ -1891,13 +1903,13 @@
         <v>0</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>124160169</v>
+        <v>125011562</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>0</v>
@@ -1906,10 +1918,10 @@
         <v>22</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>25</v>
@@ -1928,7 +1940,7 @@
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
       <c r="S18" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="T18" s="1" t="s">
         <v>30</v>
@@ -1945,44 +1957,44 @@
         <v>0</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>123314046</v>
+        <v>124160169</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>79</v>
+        <v>26</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
       <c r="R19" s="1"/>
       <c r="S19" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="T19" s="1" t="s">
         <v>30</v>
@@ -1999,44 +2011,44 @@
         <v>0</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>121807623</v>
+        <v>123314046</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H20" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>27</v>
+        <v>85</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
       <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
       <c r="S20" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="T20" s="1" t="s">
         <v>30</v>
@@ -2053,25 +2065,25 @@
         <v>0</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>124190641</v>
+        <v>121807623</v>
       </c>
       <c r="G21" s="1" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>25</v>
@@ -2090,7 +2102,7 @@
       <c r="Q21" s="1"/>
       <c r="R21" s="1"/>
       <c r="S21" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="T21" s="1" t="s">
         <v>30</v>
@@ -2107,44 +2119,44 @@
         <v>0</v>
       </c>
       <c r="D22" s="1" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>123221220</v>
+        <v>124190641</v>
       </c>
       <c r="G22" s="1" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>24</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>79</v>
+        <v>26</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
       <c r="R22" s="1"/>
       <c r="S22" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="T22" s="1" t="s">
         <v>30</v>
@@ -2161,34 +2173,34 @@
         <v>0</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F23" s="1" t="n">
-        <v>123965574</v>
+        <v>123221220</v>
       </c>
       <c r="G23" s="1" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H23" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="N23" s="1" t="s">
         <v>28</v>
@@ -2198,7 +2210,7 @@
       <c r="Q23" s="1"/>
       <c r="R23" s="1"/>
       <c r="S23" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="T23" s="1" t="s">
         <v>30</v>
@@ -2215,34 +2227,34 @@
         <v>0</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>122691466</v>
+        <v>123965574</v>
       </c>
       <c r="G24" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M24" s="1" t="s">
-        <v>27</v>
+        <v>85</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>28</v>
@@ -2252,7 +2264,7 @@
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
       <c r="S24" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="T24" s="1" t="s">
         <v>30</v>
@@ -2269,22 +2281,22 @@
         <v>0</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>120133451</v>
+        <v>122691466</v>
       </c>
       <c r="G25" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H25" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>24</v>
@@ -2299,14 +2311,14 @@
         <v>27</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
       <c r="S25" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="T25" s="1" t="s">
         <v>30</v>
@@ -2323,22 +2335,22 @@
         <v>0</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F26" s="1" t="n">
-        <v>123684162</v>
+        <v>120133451</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>24</v>
@@ -2353,14 +2365,14 @@
         <v>27</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
       <c r="S26" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="T26" s="1" t="s">
         <v>30</v>
@@ -2377,44 +2389,44 @@
         <v>0</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F27" s="1" t="n">
-        <v>124196707</v>
+        <v>123684162</v>
       </c>
       <c r="G27" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>79</v>
+        <v>26</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
       <c r="R27" s="1"/>
       <c r="S27" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="T27" s="1" t="s">
         <v>30</v>
@@ -2431,34 +2443,34 @@
         <v>0</v>
       </c>
       <c r="D28" s="1" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>121793748</v>
+        <v>124196707</v>
       </c>
       <c r="G28" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H28" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M28" s="1" t="s">
-        <v>27</v>
+        <v>85</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="N28" s="1" t="s">
         <v>28</v>
@@ -2468,7 +2480,7 @@
       <c r="Q28" s="1"/>
       <c r="R28" s="1"/>
       <c r="S28" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="T28" s="1" t="s">
         <v>30</v>
@@ -2485,44 +2497,44 @@
         <v>0</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>59</v>
+        <v>120</v>
       </c>
       <c r="F29" s="1" t="n">
-        <v>123898781</v>
+        <v>121793748</v>
       </c>
       <c r="G29" s="1" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>60</v>
+        <v>121</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>118</v>
+        <v>25</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M29" s="2" t="s">
-        <v>118</v>
+        <v>26</v>
+      </c>
+      <c r="M29" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
       <c r="R29" s="1"/>
       <c r="S29" s="1" t="s">
-        <v>63</v>
+        <v>122</v>
       </c>
       <c r="T29" s="1" t="s">
         <v>30</v>
@@ -2539,44 +2551,44 @@
         <v>0</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>120</v>
+        <v>64</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>122147393</v>
+        <v>123898781</v>
       </c>
       <c r="G30" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H30" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>121</v>
+        <v>65</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M30" s="1" t="s">
-        <v>27</v>
+        <v>124</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>122</v>
+        <v>67</v>
       </c>
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
       <c r="R30" s="1"/>
       <c r="S30" s="1" t="s">
-        <v>123</v>
+        <v>68</v>
       </c>
       <c r="T30" s="1" t="s">
         <v>30</v>
@@ -2584,7 +2596,7 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="n">
-        <v>300747284</v>
+        <v>300747283</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>20</v>
@@ -2593,22 +2605,22 @@
         <v>0</v>
       </c>
       <c r="D31" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F31" s="1" t="n">
+        <v>122147393</v>
+      </c>
+      <c r="G31" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F31" s="1" t="n">
-        <v>123293610</v>
-      </c>
-      <c r="G31" s="1" t="n">
-        <v>8</v>
-      </c>
       <c r="H31" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>24</v>
@@ -2623,14 +2635,14 @@
         <v>27</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="O31" s="1"/>
       <c r="P31" s="1"/>
       <c r="Q31" s="1"/>
       <c r="R31" s="1"/>
       <c r="S31" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="T31" s="1" t="s">
         <v>30</v>
@@ -2647,37 +2659,37 @@
         <v>0</v>
       </c>
       <c r="D32" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>123302910</v>
+        <v>123293610</v>
       </c>
       <c r="G32" s="1" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H32" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>129</v>
+        <v>25</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>129</v>
+        <v>26</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="O32" s="1"/>
       <c r="P32" s="1"/>
@@ -2701,16 +2713,16 @@
         <v>0</v>
       </c>
       <c r="D33" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>131</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>123312340</v>
+        <v>123302910</v>
       </c>
       <c r="G33" s="1" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H33" s="1" t="s">
         <v>22</v>
@@ -2719,26 +2731,26 @@
         <v>132</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>25</v>
+        <v>133</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M33" s="1" t="s">
-        <v>27</v>
+        <v>124</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>133</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>133</v>
+        <v>67</v>
       </c>
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
       <c r="Q33" s="1"/>
       <c r="R33" s="1"/>
       <c r="S33" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="T33" s="1" t="s">
         <v>30</v>
@@ -2755,22 +2767,22 @@
         <v>0</v>
       </c>
       <c r="D34" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F34" s="1" t="n">
-        <v>114842765</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>36</v>
+        <v>123312340</v>
+      </c>
+      <c r="G34" s="1" t="n">
+        <v>3</v>
       </c>
       <c r="H34" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>24</v>
@@ -2785,14 +2797,14 @@
         <v>27</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>33</v>
+        <v>137</v>
       </c>
       <c r="O34" s="1"/>
       <c r="P34" s="1"/>
       <c r="Q34" s="1"/>
       <c r="R34" s="1"/>
       <c r="S34" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="T34" s="1" t="s">
         <v>30</v>
@@ -2809,22 +2821,22 @@
         <v>0</v>
       </c>
       <c r="D35" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F35" s="1" t="n">
-        <v>122947435</v>
-      </c>
-      <c r="G35" s="1" t="n">
-        <v>3</v>
+        <v>114842765</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>24</v>
@@ -2839,14 +2851,14 @@
         <v>27</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>122</v>
+        <v>33</v>
       </c>
       <c r="O35" s="1"/>
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
       <c r="R35" s="1"/>
       <c r="S35" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="T35" s="1" t="s">
         <v>30</v>
@@ -2863,22 +2875,22 @@
         <v>0</v>
       </c>
       <c r="D36" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F36" s="1" t="n">
-        <v>120929761</v>
+        <v>122947435</v>
       </c>
       <c r="G36" s="1" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>24</v>
@@ -2893,14 +2905,14 @@
         <v>27</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="O36" s="1"/>
       <c r="P36" s="1"/>
       <c r="Q36" s="1"/>
       <c r="R36" s="1"/>
       <c r="S36" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T36" s="1" t="s">
         <v>30</v>
@@ -2917,22 +2929,22 @@
         <v>0</v>
       </c>
       <c r="D37" s="1" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F37" s="1" t="n">
-        <v>123051671</v>
+        <v>120929761</v>
       </c>
       <c r="G37" s="1" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H37" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>24</v>
@@ -2954,7 +2966,7 @@
       <c r="Q37" s="1"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="T37" s="1" t="s">
         <v>30</v>
@@ -2971,22 +2983,22 @@
         <v>0</v>
       </c>
       <c r="D38" s="1" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F38" s="1" t="n">
-        <v>123319101</v>
+        <v>123051671</v>
       </c>
       <c r="G38" s="1" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H38" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J38" s="2" t="s">
         <v>24</v>
@@ -3008,7 +3020,7 @@
       <c r="Q38" s="1"/>
       <c r="R38" s="1"/>
       <c r="S38" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="T38" s="1" t="s">
         <v>30</v>
@@ -3025,22 +3037,22 @@
         <v>0</v>
       </c>
       <c r="D39" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F39" s="1" t="n">
+        <v>123319101</v>
+      </c>
+      <c r="G39" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="E39" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="F39" s="1" t="n">
-        <v>124369160</v>
-      </c>
-      <c r="G39" s="1" t="n">
-        <v>8</v>
-      </c>
       <c r="H39" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>24</v>
@@ -3062,7 +3074,7 @@
       <c r="Q39" s="1"/>
       <c r="R39" s="1"/>
       <c r="S39" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="T39" s="1" t="s">
         <v>30</v>
@@ -3079,22 +3091,22 @@
         <v>0</v>
       </c>
       <c r="D40" s="1" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F40" s="1" t="n">
-        <v>121356744</v>
+        <v>124369160</v>
       </c>
       <c r="G40" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H40" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>24</v>
@@ -3116,7 +3128,7 @@
       <c r="Q40" s="1"/>
       <c r="R40" s="1"/>
       <c r="S40" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="T40" s="1" t="s">
         <v>30</v>
@@ -3133,22 +3145,22 @@
         <v>0</v>
       </c>
       <c r="D41" s="1" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F41" s="1" t="n">
-        <v>122407121</v>
+        <v>121356744</v>
       </c>
       <c r="G41" s="1" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H41" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>24</v>
@@ -3170,7 +3182,7 @@
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
       <c r="S41" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="T41" s="1" t="s">
         <v>30</v>
@@ -3187,22 +3199,22 @@
         <v>0</v>
       </c>
       <c r="D42" s="1" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F42" s="1" t="n">
-        <v>123258153</v>
+        <v>122407121</v>
       </c>
       <c r="G42" s="1" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>24</v>
@@ -3224,7 +3236,7 @@
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
       <c r="S42" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T42" s="1" t="s">
         <v>30</v>
@@ -3241,22 +3253,22 @@
         <v>0</v>
       </c>
       <c r="D43" s="1" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F43" s="1" t="n">
-        <v>122888452</v>
+        <v>123258153</v>
       </c>
       <c r="G43" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H43" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>24</v>
@@ -3278,7 +3290,7 @@
       <c r="Q43" s="1"/>
       <c r="R43" s="1"/>
       <c r="S43" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="T43" s="1" t="s">
         <v>30</v>
@@ -3295,22 +3307,22 @@
         <v>0</v>
       </c>
       <c r="D44" s="1" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F44" s="1" t="n">
-        <v>123802186</v>
+        <v>122888452</v>
       </c>
       <c r="G44" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H44" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>113</v>
+        <v>166</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>24</v>
@@ -3325,14 +3337,14 @@
         <v>27</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="O44" s="1"/>
       <c r="P44" s="1"/>
       <c r="Q44" s="1"/>
       <c r="R44" s="1"/>
       <c r="S44" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T44" s="1" t="s">
         <v>30</v>
@@ -3349,22 +3361,22 @@
         <v>0</v>
       </c>
       <c r="D45" s="1" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F45" s="1" t="n">
-        <v>124068081</v>
+        <v>123802186</v>
       </c>
       <c r="G45" s="1" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H45" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>167</v>
+        <v>118</v>
       </c>
       <c r="J45" s="2" t="s">
         <v>24</v>
@@ -3379,14 +3391,14 @@
         <v>27</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>122</v>
+        <v>28</v>
       </c>
       <c r="O45" s="1"/>
       <c r="P45" s="1"/>
       <c r="Q45" s="1"/>
       <c r="R45" s="1"/>
       <c r="S45" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="T45" s="1" t="s">
         <v>30</v>
@@ -3403,22 +3415,22 @@
         <v>0</v>
       </c>
       <c r="D46" s="1" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F46" s="1" t="n">
-        <v>124017729</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>36</v>
+        <v>124068081</v>
+      </c>
+      <c r="G46" s="1" t="n">
+        <v>8</v>
       </c>
       <c r="H46" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J46" s="2" t="s">
         <v>24</v>
@@ -3433,14 +3445,14 @@
         <v>27</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
       <c r="Q46" s="1"/>
       <c r="R46" s="1"/>
       <c r="S46" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T46" s="1" t="s">
         <v>30</v>
@@ -3457,22 +3469,22 @@
         <v>0</v>
       </c>
       <c r="D47" s="1" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F47" s="1" t="n">
-        <v>123660665</v>
-      </c>
-      <c r="G47" s="1" t="n">
-        <v>6</v>
+        <v>124017729</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="H47" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J47" s="2" t="s">
         <v>24</v>
@@ -3494,7 +3506,7 @@
       <c r="Q47" s="1"/>
       <c r="R47" s="1"/>
       <c r="S47" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T47" s="1" t="s">
         <v>30</v>
@@ -3511,22 +3523,22 @@
         <v>0</v>
       </c>
       <c r="D48" s="1" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F48" s="1" t="n">
-        <v>123625859</v>
+        <v>123660665</v>
       </c>
       <c r="G48" s="1" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H48" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>24</v>
@@ -3548,7 +3560,7 @@
       <c r="Q48" s="1"/>
       <c r="R48" s="1"/>
       <c r="S48" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="T48" s="1" t="s">
         <v>30</v>
@@ -3565,25 +3577,25 @@
         <v>0</v>
       </c>
       <c r="D49" s="1" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F49" s="1" t="n">
-        <v>123235406</v>
+        <v>123625859</v>
       </c>
       <c r="G49" s="1" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H49" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>25</v>
@@ -3602,7 +3614,7 @@
       <c r="Q49" s="1"/>
       <c r="R49" s="1"/>
       <c r="S49" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="T49" s="1" t="s">
         <v>30</v>
@@ -3619,44 +3631,44 @@
         <v>0</v>
       </c>
       <c r="D50" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F50" s="1" t="n">
-        <v>122306181</v>
+        <v>123235406</v>
       </c>
       <c r="G50" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H50" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>118</v>
+        <v>25</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M50" s="2" t="s">
-        <v>118</v>
+        <v>26</v>
+      </c>
+      <c r="M50" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="O50" s="1"/>
       <c r="P50" s="1"/>
       <c r="Q50" s="1"/>
       <c r="R50" s="1"/>
       <c r="S50" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="T50" s="1" t="s">
         <v>30</v>
@@ -3664,7 +3676,7 @@
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="n">
-        <v>300747285</v>
+        <v>300747284</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>20</v>
@@ -3673,44 +3685,44 @@
         <v>0</v>
       </c>
       <c r="D51" s="1" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F51" s="1" t="n">
-        <v>122817084</v>
+        <v>122306181</v>
       </c>
       <c r="G51" s="1" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H51" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M51" s="1" t="s">
-        <v>27</v>
+        <v>124</v>
+      </c>
+      <c r="M51" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
       <c r="Q51" s="1"/>
       <c r="R51" s="1"/>
       <c r="S51" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="T51" s="1" t="s">
         <v>30</v>
@@ -3727,25 +3739,25 @@
         <v>0</v>
       </c>
       <c r="D52" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>127</v>
+        <v>187</v>
       </c>
       <c r="F52" s="1" t="n">
-        <v>123302910</v>
+        <v>122817084</v>
       </c>
       <c r="G52" s="1" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H52" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>128</v>
+        <v>188</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>186</v>
+        <v>24</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>25</v>
@@ -3757,14 +3769,14 @@
         <v>27</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="O52" s="1"/>
       <c r="P52" s="1"/>
       <c r="Q52" s="1"/>
       <c r="R52" s="1"/>
       <c r="S52" s="1" t="s">
-        <v>130</v>
+        <v>189</v>
       </c>
       <c r="T52" s="1" t="s">
         <v>30</v>
@@ -3781,25 +3793,25 @@
         <v>0</v>
       </c>
       <c r="D53" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>187</v>
+        <v>131</v>
       </c>
       <c r="F53" s="1" t="n">
-        <v>123684018</v>
+        <v>123302910</v>
       </c>
       <c r="G53" s="1" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H53" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>188</v>
+        <v>132</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>61</v>
+        <v>190</v>
       </c>
       <c r="K53" s="2" t="s">
         <v>25</v>
@@ -3811,14 +3823,14 @@
         <v>27</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="O53" s="1"/>
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
       <c r="R53" s="1"/>
       <c r="S53" s="1" t="s">
-        <v>189</v>
+        <v>134</v>
       </c>
       <c r="T53" s="1" t="s">
         <v>30</v>
@@ -3835,25 +3847,25 @@
         <v>0</v>
       </c>
       <c r="D54" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F54" s="1" t="n">
-        <v>121014315</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>36</v>
+        <v>123684018</v>
+      </c>
+      <c r="G54" s="1" t="n">
+        <v>5</v>
       </c>
       <c r="H54" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="K54" s="2" t="s">
         <v>25</v>
@@ -3872,7 +3884,7 @@
       <c r="Q54" s="1"/>
       <c r="R54" s="1"/>
       <c r="S54" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="T54" s="1" t="s">
         <v>30</v>
@@ -3889,22 +3901,22 @@
         <v>0</v>
       </c>
       <c r="D55" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F55" s="1" t="n">
-        <v>122271146</v>
-      </c>
-      <c r="G55" s="1" t="n">
-        <v>1</v>
+        <v>121014315</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="H55" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J55" s="2" t="s">
         <v>24</v>
@@ -3919,14 +3931,14 @@
         <v>27</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="O55" s="1"/>
       <c r="P55" s="1"/>
       <c r="Q55" s="1"/>
       <c r="R55" s="1"/>
       <c r="S55" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="T55" s="1" t="s">
         <v>30</v>
@@ -3943,22 +3955,22 @@
         <v>0</v>
       </c>
       <c r="D56" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F56" s="1" t="n">
-        <v>124017673</v>
+        <v>122271146</v>
       </c>
       <c r="G56" s="1" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H56" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>170</v>
+        <v>198</v>
       </c>
       <c r="J56" s="2" t="s">
         <v>24</v>
@@ -3973,14 +3985,14 @@
         <v>27</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="O56" s="1"/>
       <c r="P56" s="1"/>
       <c r="Q56" s="1"/>
       <c r="R56" s="1"/>
       <c r="S56" s="1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="T56" s="1" t="s">
         <v>30</v>
@@ -3997,22 +4009,22 @@
         <v>0</v>
       </c>
       <c r="D57" s="1" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F57" s="1" t="n">
-        <v>122304525</v>
+        <v>124017673</v>
       </c>
       <c r="G57" s="1" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H57" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>199</v>
+        <v>174</v>
       </c>
       <c r="J57" s="2" t="s">
         <v>24</v>
@@ -4027,14 +4039,14 @@
         <v>27</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="O57" s="1"/>
       <c r="P57" s="1"/>
       <c r="Q57" s="1"/>
       <c r="R57" s="1"/>
       <c r="S57" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="T57" s="1" t="s">
         <v>30</v>
@@ -4051,22 +4063,22 @@
         <v>0</v>
       </c>
       <c r="D58" s="1" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F58" s="1" t="n">
-        <v>122410258</v>
+        <v>122304525</v>
       </c>
       <c r="G58" s="1" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H58" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J58" s="2" t="s">
         <v>24</v>
@@ -4081,14 +4093,14 @@
         <v>27</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="O58" s="1"/>
       <c r="P58" s="1"/>
       <c r="Q58" s="1"/>
       <c r="R58" s="1"/>
       <c r="S58" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="T58" s="1" t="s">
         <v>30</v>
@@ -4105,22 +4117,22 @@
         <v>0</v>
       </c>
       <c r="D59" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F59" s="1" t="n">
-        <v>121440175</v>
+        <v>122410258</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H59" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J59" s="2" t="s">
         <v>24</v>
@@ -4135,14 +4147,14 @@
         <v>27</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="O59" s="1"/>
       <c r="P59" s="1"/>
       <c r="Q59" s="1"/>
       <c r="R59" s="1"/>
       <c r="S59" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="T59" s="1" t="s">
         <v>30</v>
@@ -4159,22 +4171,22 @@
         <v>0</v>
       </c>
       <c r="D60" s="1" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F60" s="1" t="n">
-        <v>120617922</v>
+        <v>121440175</v>
       </c>
       <c r="G60" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H60" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J60" s="2" t="s">
         <v>24</v>
@@ -4189,14 +4201,14 @@
         <v>27</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="O60" s="1"/>
       <c r="P60" s="1"/>
       <c r="Q60" s="1"/>
       <c r="R60" s="1"/>
       <c r="S60" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="T60" s="1" t="s">
         <v>30</v>
@@ -4213,22 +4225,22 @@
         <v>0</v>
       </c>
       <c r="D61" s="1" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F61" s="1" t="n">
-        <v>125682919</v>
+        <v>120617922</v>
       </c>
       <c r="G61" s="1" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H61" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J61" s="2" t="s">
         <v>24</v>
@@ -4243,7 +4255,7 @@
         <v>27</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>212</v>
+        <v>33</v>
       </c>
       <c r="O61" s="1"/>
       <c r="P61" s="1"/>
@@ -4267,25 +4279,25 @@
         <v>0</v>
       </c>
       <c r="D62" s="1" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>180</v>
+        <v>214</v>
       </c>
       <c r="F62" s="1" t="n">
-        <v>122306181</v>
+        <v>125682919</v>
       </c>
       <c r="G62" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H62" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>181</v>
+        <v>215</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="K62" s="2" t="s">
         <v>25</v>
@@ -4297,14 +4309,14 @@
         <v>27</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>62</v>
+        <v>216</v>
       </c>
       <c r="O62" s="1"/>
       <c r="P62" s="1"/>
       <c r="Q62" s="1"/>
       <c r="R62" s="1"/>
       <c r="S62" s="1" t="s">
-        <v>182</v>
+        <v>217</v>
       </c>
       <c r="T62" s="1" t="s">
         <v>30</v>
@@ -4321,25 +4333,25 @@
         <v>0</v>
       </c>
       <c r="D63" s="1" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>214</v>
+        <v>184</v>
       </c>
       <c r="F63" s="1" t="n">
-        <v>124894646</v>
+        <v>122306181</v>
       </c>
       <c r="G63" s="1" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H63" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>215</v>
+        <v>185</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="K63" s="2" t="s">
         <v>25</v>
@@ -4351,14 +4363,14 @@
         <v>27</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="O63" s="1"/>
       <c r="P63" s="1"/>
       <c r="Q63" s="1"/>
       <c r="R63" s="1"/>
       <c r="S63" s="1" t="s">
-        <v>216</v>
+        <v>186</v>
       </c>
       <c r="T63" s="1" t="s">
         <v>30</v>
@@ -4366,7 +4378,7 @@
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="n">
-        <v>300747287</v>
+        <v>300747285</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>20</v>
@@ -4375,22 +4387,22 @@
         <v>0</v>
       </c>
       <c r="D64" s="1" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F64" s="1" t="n">
-        <v>120617914</v>
+        <v>124894646</v>
       </c>
       <c r="G64" s="1" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H64" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="J64" s="2" t="s">
         <v>24</v>
@@ -4405,14 +4417,14 @@
         <v>27</v>
       </c>
       <c r="N64" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="O64" s="1"/>
       <c r="P64" s="1"/>
       <c r="Q64" s="1"/>
       <c r="R64" s="1"/>
       <c r="S64" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="T64" s="1" t="s">
         <v>30</v>
@@ -4429,22 +4441,22 @@
         <v>0</v>
       </c>
       <c r="D65" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F65" s="1" t="n">
-        <v>123230596</v>
+        <v>120617914</v>
       </c>
       <c r="G65" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H65" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="J65" s="2" t="s">
         <v>24</v>
@@ -4459,7 +4471,7 @@
         <v>27</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>221</v>
+        <v>33</v>
       </c>
       <c r="O65" s="1"/>
       <c r="P65" s="1"/>
@@ -4483,16 +4495,16 @@
         <v>0</v>
       </c>
       <c r="D66" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>223</v>
       </c>
       <c r="F66" s="1" t="n">
-        <v>124373914</v>
+        <v>123230596</v>
       </c>
       <c r="G66" s="1" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H66" s="1" t="s">
         <v>22</v>
@@ -4513,14 +4525,14 @@
         <v>27</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>33</v>
+        <v>225</v>
       </c>
       <c r="O66" s="1"/>
       <c r="P66" s="1"/>
       <c r="Q66" s="1"/>
       <c r="R66" s="1"/>
       <c r="S66" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="T66" s="1" t="s">
         <v>30</v>
@@ -4537,22 +4549,22 @@
         <v>0</v>
       </c>
       <c r="D67" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F67" s="1" t="n">
-        <v>114842803</v>
+        <v>124373914</v>
       </c>
       <c r="G67" s="1" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H67" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I67" s="2" t="s">
-        <v>135</v>
+        <v>228</v>
       </c>
       <c r="J67" s="2" t="s">
         <v>24</v>
@@ -4574,7 +4586,7 @@
       <c r="Q67" s="1"/>
       <c r="R67" s="1"/>
       <c r="S67" s="1" t="s">
-        <v>136</v>
+        <v>229</v>
       </c>
       <c r="T67" s="1" t="s">
         <v>30</v>
@@ -4591,22 +4603,22 @@
         <v>0</v>
       </c>
       <c r="D68" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F68" s="1" t="n">
-        <v>123714593</v>
+        <v>114842803</v>
       </c>
       <c r="G68" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H68" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>188</v>
+        <v>139</v>
       </c>
       <c r="J68" s="2" t="s">
         <v>24</v>
@@ -4621,14 +4633,14 @@
         <v>27</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="O68" s="1"/>
       <c r="P68" s="1"/>
       <c r="Q68" s="1"/>
       <c r="R68" s="1"/>
       <c r="S68" s="1" t="s">
-        <v>228</v>
+        <v>140</v>
       </c>
       <c r="T68" s="1" t="s">
         <v>30</v>
@@ -4645,22 +4657,22 @@
         <v>0</v>
       </c>
       <c r="D69" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F69" s="1" t="n">
-        <v>121261324</v>
+        <v>123714593</v>
       </c>
       <c r="G69" s="1" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H69" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>116</v>
+        <v>192</v>
       </c>
       <c r="J69" s="2" t="s">
         <v>24</v>
@@ -4675,14 +4687,14 @@
         <v>27</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="O69" s="1"/>
       <c r="P69" s="1"/>
       <c r="Q69" s="1"/>
       <c r="R69" s="1"/>
       <c r="S69" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="T69" s="1" t="s">
         <v>30</v>
@@ -4699,22 +4711,22 @@
         <v>0</v>
       </c>
       <c r="D70" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F70" s="1" t="n">
+        <v>121261324</v>
+      </c>
+      <c r="G70" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="E70" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="F70" s="1" t="n">
-        <v>123690731</v>
-      </c>
-      <c r="G70" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="H70" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I70" s="2" t="s">
-        <v>232</v>
+        <v>121</v>
       </c>
       <c r="J70" s="2" t="s">
         <v>24</v>
@@ -4736,7 +4748,7 @@
       <c r="Q70" s="1"/>
       <c r="R70" s="1"/>
       <c r="S70" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="T70" s="1" t="s">
         <v>30</v>
@@ -4753,22 +4765,22 @@
         <v>0</v>
       </c>
       <c r="D71" s="1" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F71" s="1" t="n">
-        <v>121440193</v>
+        <v>123690731</v>
       </c>
       <c r="G71" s="1" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H71" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="J71" s="2" t="s">
         <v>24</v>
@@ -4783,16 +4795,70 @@
         <v>27</v>
       </c>
       <c r="N71" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="O71" s="1"/>
       <c r="P71" s="1"/>
       <c r="Q71" s="1"/>
       <c r="R71" s="1"/>
       <c r="S71" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="T71" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="n">
+        <v>300747287</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C72" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="F72" s="1" t="n">
+        <v>121440193</v>
+      </c>
+      <c r="G72" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K72" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L72" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M72" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N72" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O72" s="1"/>
+      <c r="P72" s="1"/>
+      <c r="Q72" s="1"/>
+      <c r="R72" s="1"/>
+      <c r="S72" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="T72" s="1" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>